<commit_message>
Add accordion-faq block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 41
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article-text.report.xlsx
+++ b/tools/importer/reports/import-article-text.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="125">
   <si>
     <t>_reportFile</t>
   </si>
@@ -82,6 +82,27 @@
     <t>https://www.dunkincreamer.com/</t>
   </si>
   <si>
+    <t>where-to-buy-dunkin-creamer.report.json</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>where-to-buy-dunkin-creamer</t>
+  </si>
+  <si>
+    <t>recipe-detail</t>
+  </si>
+  <si>
+    <t>2026-09-23T09:06:16.437Z</t>
+  </si>
+  <si>
+    <t>Where To Buy Dunkin’® Creamer</t>
+  </si>
+  <si>
+    <t>https://www.dunkincreamer.com/where-to-buy-dunkin-creamer/</t>
+  </si>
+  <si>
     <t>author/danoneitccadmin.report.json</t>
   </si>
   <si>
@@ -103,6 +124,21 @@
     <t>https://www.dunkincreamer.com/author/danoneitccadmin/</t>
   </si>
   <si>
+    <t>category/uncategorized.report.json</t>
+  </si>
+  <si>
+    <t>category/uncategorized</t>
+  </si>
+  <si>
+    <t>2026-09-23T09:05:20.158Z</t>
+  </si>
+  <si>
+    <t>Uncategorized Archives - DunkinCreamer</t>
+  </si>
+  <si>
+    <t>https://www.dunkincreamer.com/category/uncategorized/</t>
+  </si>
+  <si>
     <t>coffee-creamer/coffee-creamer.report.json</t>
   </si>
   <si>
@@ -115,7 +151,7 @@
     <t>product-detail</t>
   </si>
   <si>
-    <t>2026-09-23T08:44:56.745Z</t>
+    <t>2026-09-23T14:09:15.414Z</t>
   </si>
   <si>
     <t>coffee-creamer Archives - DunkinCreamer</t>
@@ -124,6 +160,66 @@
     <t>https://www.dunkincreamer.com/coffee-creamer/coffee-creamer/</t>
   </si>
   <si>
+    <t>coffee-creamer/extra-extra-creamer.report.json</t>
+  </si>
+  <si>
+    <t>coffee-creamer/extra-extra-creamer</t>
+  </si>
+  <si>
+    <t>2026-09-23T09:02:41.242Z</t>
+  </si>
+  <si>
+    <t>Dunkin’® Extra Extra Coffee Creamer</t>
+  </si>
+  <si>
+    <t>https://www.dunkincreamer.com/coffee-creamer/extra-extra-creamer/</t>
+  </si>
+  <si>
+    <t>coffee-creamer/pumpkin-munchkin.report.json</t>
+  </si>
+  <si>
+    <t>coffee-creamer/pumpkin-munchkin</t>
+  </si>
+  <si>
+    <t>2026-09-23T09:03:34.507Z</t>
+  </si>
+  <si>
+    <t>ITS BACK! PUMPKIN MUNCHKIN COFFEE CREAMER - Dunkin’ Creamer</t>
+  </si>
+  <si>
+    <t>https://www.dunkincreamer.com/coffee-creamer/pumpkin-munchkin/</t>
+  </si>
+  <si>
+    <t>cold-foam-creamer/extra-extra-cold-foam-creamer.report.json</t>
+  </si>
+  <si>
+    <t>cold-foam-creamer/extra-extra-cold-foam-creamer</t>
+  </si>
+  <si>
+    <t>2026-09-23T09:04:28.615Z</t>
+  </si>
+  <si>
+    <t>Dunkin’® Extra Extra Cold Foam Creamer</t>
+  </si>
+  <si>
+    <t>https://www.dunkincreamer.com/cold-foam-creamer/extra-extra-cold-foam-creamer/</t>
+  </si>
+  <si>
+    <t>learn-more/about-dunkins.report.json</t>
+  </si>
+  <si>
+    <t>learn-more/about-dunkins</t>
+  </si>
+  <si>
+    <t>2026-09-23T09:05:12.527Z</t>
+  </si>
+  <si>
+    <t>About Dunkin’® Coffee Creamers</t>
+  </si>
+  <si>
+    <t>https://www.dunkincreamer.com/learn-more/about-dunkins/</t>
+  </si>
+  <si>
     <t>learn-more/coffee-creamer-recipes.report.json</t>
   </si>
   <si>
@@ -178,7 +274,7 @@
     <t>article-text</t>
   </si>
   <si>
-    <t>2026-09-23T08:45:46.865Z</t>
+    <t>2026-09-23T14:09:31.264Z</t>
   </si>
   <si>
     <t>Dunkin’® Creamers Pressroom</t>
@@ -187,6 +283,30 @@
     <t>https://www.dunkincreamer.com/learn-more/pressroom/</t>
   </si>
   <si>
+    <t>learn-more/coffee-creamer-recipes/ball-game-blender.report.json</t>
+  </si>
+  <si>
+    <t>learn-more/coffee-creamer-recipes/ball-game-blender</t>
+  </si>
+  <si>
+    <t>2026-09-23T09:05:30.188Z</t>
+  </si>
+  <si>
+    <t>https://www.dunkincreamer.com/learn-more/coffee-creamer-recipes/ball-game-blender/</t>
+  </si>
+  <si>
+    <t>learn-more/coffee-creamer-recipes/blueberry-muffins.report.json</t>
+  </si>
+  <si>
+    <t>learn-more/coffee-creamer-recipes/blueberry-muffins</t>
+  </si>
+  <si>
+    <t>2026-09-23T09:05:38.166Z</t>
+  </si>
+  <si>
+    <t>https://www.dunkincreamer.com/learn-more/coffee-creamer-recipes/blueberry-muffins/</t>
+  </si>
+  <si>
     <t>learn-more/coffee-creamer-recipes/coconut-cream-pie-blender.report.json</t>
   </si>
   <si>
@@ -196,9 +316,6 @@
     <t>learn-more/coffee-creamer-recipes/coconut-cream-pie-blender</t>
   </si>
   <si>
-    <t>recipe-detail</t>
-  </si>
-  <si>
     <t>2026-09-23T08:45:30.455Z</t>
   </si>
   <si>
@@ -206,6 +323,48 @@
   </si>
   <si>
     <t>https://www.dunkincreamer.com/learn-more/coffee-creamer-recipes/coconut-cream-pie-blender/</t>
+  </si>
+  <si>
+    <t>learn-more/coffee-creamer-recipes/easy-tres-leches-cake.report.json</t>
+  </si>
+  <si>
+    <t>learn-more/coffee-creamer-recipes/easy-tres-leches-cake</t>
+  </si>
+  <si>
+    <t>2026-09-23T09:05:57.380Z</t>
+  </si>
+  <si>
+    <t>Easy Tres Leches Cake Recipe with Dunkin’® Creamers</t>
+  </si>
+  <si>
+    <t>https://www.dunkincreamer.com/learn-more/coffee-creamer-recipes/easy-tres-leches-cake/</t>
+  </si>
+  <si>
+    <t>learn-more/coffee-creamer-recipes/english-toffee-coffee.report.json</t>
+  </si>
+  <si>
+    <t>learn-more/coffee-creamer-recipes/english-toffee-coffee</t>
+  </si>
+  <si>
+    <t>2026-09-23T09:05:46.818Z</t>
+  </si>
+  <si>
+    <t>https://www.dunkincreamer.com/learn-more/coffee-creamer-recipes/english-toffee-coffee/</t>
+  </si>
+  <si>
+    <t>learn-more/coffee-creamer-recipes/latte-maximus.report.json</t>
+  </si>
+  <si>
+    <t>learn-more/coffee-creamer-recipes/latte-maximus</t>
+  </si>
+  <si>
+    <t>2026-09-23T09:06:05.893Z</t>
+  </si>
+  <si>
+    <t>Latte Maximus Recipe with Dunkin’® Creamer</t>
+  </si>
+  <si>
+    <t>https://www.dunkincreamer.com/learn-more/coffee-creamer-recipes/latte-maximus/</t>
   </si>
   <si>
     <t>2020/02/28/hello-world.report.json</t>
@@ -615,7 +774,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -759,129 +918,415 @@
         <v>37</v>
       </c>
       <c r="B6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" t="s">
         <v>38</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" t="s">
         <v>39</v>
       </c>
-      <c r="D6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="G6" t="s">
         <v>40</v>
       </c>
-      <c r="F6" t="s">
+      <c r="H6" t="s">
         <v>41</v>
-      </c>
-      <c r="G6" t="s">
-        <v>42</v>
-      </c>
-      <c r="H6" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" t="s">
         <v>44</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
         <v>45</v>
       </c>
-      <c r="C7" t="s">
+      <c r="F7" t="s">
         <v>46</v>
       </c>
-      <c r="D7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" t="s">
+      <c r="G7" t="s">
         <v>47</v>
       </c>
-      <c r="F7" t="s">
+      <c r="H7" t="s">
         <v>48</v>
-      </c>
-      <c r="G7" t="s">
-        <v>49</v>
-      </c>
-      <c r="H7" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" t="s">
         <v>51</v>
       </c>
-      <c r="B8" t="s">
+      <c r="G8" t="s">
         <v>52</v>
       </c>
-      <c r="C8" t="s">
+      <c r="H8" t="s">
         <v>53</v>
-      </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
-        <v>54</v>
-      </c>
-      <c r="F8" t="s">
-        <v>55</v>
-      </c>
-      <c r="G8" t="s">
-        <v>56</v>
-      </c>
-      <c r="H8" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s">
+        <v>55</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" t="s">
+        <v>56</v>
+      </c>
+      <c r="G9" t="s">
+        <v>57</v>
+      </c>
+      <c r="H9" t="s">
         <v>58</v>
-      </c>
-      <c r="B9" t="s">
-        <v>59</v>
-      </c>
-      <c r="C9" t="s">
-        <v>60</v>
-      </c>
-      <c r="D9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" t="s">
-        <v>61</v>
-      </c>
-      <c r="F9" t="s">
-        <v>62</v>
-      </c>
-      <c r="G9" t="s">
-        <v>63</v>
-      </c>
-      <c r="H9" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" t="s">
+        <v>61</v>
+      </c>
+      <c r="G10" t="s">
+        <v>62</v>
+      </c>
+      <c r="H10" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" t="s">
         <v>65</v>
       </c>
-      <c r="B10" t="s">
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" t="s">
         <v>66</v>
       </c>
-      <c r="C10" t="s">
+      <c r="G11" t="s">
         <v>67</v>
       </c>
-      <c r="D10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" t="s">
+      <c r="H11" t="s">
         <v>68</v>
       </c>
-      <c r="F10" t="s">
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>69</v>
       </c>
-      <c r="G10" t="s">
+      <c r="B12" t="s">
         <v>70</v>
       </c>
-      <c r="H10" t="s">
+      <c r="C12" t="s">
         <v>71</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>72</v>
+      </c>
+      <c r="F12" t="s">
+        <v>73</v>
+      </c>
+      <c r="G12" t="s">
+        <v>74</v>
+      </c>
+      <c r="H12" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" t="s">
+        <v>77</v>
+      </c>
+      <c r="C13" t="s">
+        <v>78</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>79</v>
+      </c>
+      <c r="F13" t="s">
+        <v>80</v>
+      </c>
+      <c r="G13" t="s">
+        <v>81</v>
+      </c>
+      <c r="H13" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>83</v>
+      </c>
+      <c r="B14" t="s">
+        <v>84</v>
+      </c>
+      <c r="C14" t="s">
+        <v>85</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>86</v>
+      </c>
+      <c r="F14" t="s">
+        <v>87</v>
+      </c>
+      <c r="G14" t="s">
+        <v>88</v>
+      </c>
+      <c r="H14" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B15" t="s">
+        <v>70</v>
+      </c>
+      <c r="C15" t="s">
+        <v>91</v>
+      </c>
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
+        <v>72</v>
+      </c>
+      <c r="F15" t="s">
+        <v>92</v>
+      </c>
+      <c r="G15" t="s">
+        <v>74</v>
+      </c>
+      <c r="H15" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" t="s">
+        <v>70</v>
+      </c>
+      <c r="C16" t="s">
+        <v>95</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>72</v>
+      </c>
+      <c r="F16" t="s">
+        <v>96</v>
+      </c>
+      <c r="G16" t="s">
+        <v>74</v>
+      </c>
+      <c r="H16" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>98</v>
+      </c>
+      <c r="B17" t="s">
+        <v>99</v>
+      </c>
+      <c r="C17" t="s">
+        <v>100</v>
+      </c>
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>26</v>
+      </c>
+      <c r="F17" t="s">
+        <v>101</v>
+      </c>
+      <c r="G17" t="s">
+        <v>102</v>
+      </c>
+      <c r="H17" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>104</v>
+      </c>
+      <c r="B18" t="s">
+        <v>99</v>
+      </c>
+      <c r="C18" t="s">
+        <v>105</v>
+      </c>
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>26</v>
+      </c>
+      <c r="F18" t="s">
+        <v>106</v>
+      </c>
+      <c r="G18" t="s">
+        <v>107</v>
+      </c>
+      <c r="H18" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" t="s">
+        <v>70</v>
+      </c>
+      <c r="C19" t="s">
+        <v>110</v>
+      </c>
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" t="s">
+        <v>72</v>
+      </c>
+      <c r="F19" t="s">
+        <v>111</v>
+      </c>
+      <c r="G19" t="s">
+        <v>74</v>
+      </c>
+      <c r="H19" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>113</v>
+      </c>
+      <c r="B20" t="s">
+        <v>99</v>
+      </c>
+      <c r="C20" t="s">
+        <v>114</v>
+      </c>
+      <c r="D20" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" t="s">
+        <v>26</v>
+      </c>
+      <c r="F20" t="s">
+        <v>115</v>
+      </c>
+      <c r="G20" t="s">
+        <v>116</v>
+      </c>
+      <c r="H20" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>118</v>
+      </c>
+      <c r="B21" t="s">
+        <v>119</v>
+      </c>
+      <c r="C21" t="s">
+        <v>120</v>
+      </c>
+      <c r="D21" t="s">
+        <v>11</v>
+      </c>
+      <c r="E21" t="s">
+        <v>121</v>
+      </c>
+      <c r="F21" t="s">
+        <v>122</v>
+      </c>
+      <c r="G21" t="s">
+        <v>123</v>
+      </c>
+      <c r="H21" t="s">
+        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>